<commit_message>
Uppdated production data for Glencore and added crude ore for certain facilities
</commit_message>
<xml_diff>
--- a/data/Companies_reports/Glencore/GLEN_2024-FY_ProductionReport_tables.xlsx
+++ b/data/Companies_reports/Glencore/GLEN_2024-FY_ProductionReport_tables.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
   <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{705B2B95-2ED2-4662-AC2F-A0135E34FE9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1BCD44F5-EFD7-4CC7-AFDE-65A59B6777DA}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="24576" yWindow="1716" windowWidth="17280" windowHeight="8880" xr2:uid="{40108302-4415-4DD7-97F7-D08B79BDEF4B}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{40108302-4415-4DD7-97F7-D08B79BDEF4B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1778,6 +1778,48 @@
     <xf numFmtId="166" fontId="35" fillId="0" borderId="13" xfId="52" applyFont="1" applyBorder="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="3" xfId="45" applyFont="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="65" applyFont="1" applyBorder="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="65" applyFont="1" applyBorder="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="10" xfId="58" applyFont="1" applyBorder="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="10" xfId="68" applyFont="1" applyBorder="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="11" xfId="68" applyFont="1" applyBorder="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="10" xfId="68" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="13" xfId="65" applyFont="1" applyBorder="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="14" xfId="68" applyFont="1" applyBorder="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="15" xfId="68" applyFont="1" applyBorder="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="13" xfId="66" applyFont="1" applyBorder="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="14" xfId="68" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="15" xfId="68" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="13" xfId="56" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1787,50 +1829,8 @@
     <xf numFmtId="0" fontId="34" fillId="0" borderId="13" xfId="58" applyFont="1" applyBorder="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="65" applyFont="1" applyBorder="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="13" xfId="65" applyFont="1" applyBorder="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="56" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" xfId="65" applyFont="1" applyBorder="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="14" xfId="68" applyFont="1" applyBorder="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="15" xfId="68" applyFont="1" applyBorder="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="13" xfId="66" applyFont="1" applyBorder="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="14" xfId="68" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="15" xfId="68" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="10" xfId="58" applyFont="1" applyBorder="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="10" xfId="68" applyFont="1" applyBorder="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="11" xfId="68" applyFont="1" applyBorder="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="10" xfId="68" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="3" xfId="45" applyFont="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="73">
@@ -1921,12 +1921,8 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -2246,13 +2242,13 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:L231"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="40.109375" customWidth="1"/>
-    <col min="2" max="2" width="23.33203125" customWidth="1"/>
+    <col min="1" max="1" width="40.08984375" customWidth="1"/>
+    <col min="2" max="2" width="23.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="16.8">
+    <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -2264,7 +2260,7 @@
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
     </row>
-    <row r="2" spans="1:12" ht="16.8">
+    <row r="2" spans="1:12">
       <c r="A2" s="1" t="s">
         <v>25</v>
       </c>
@@ -2277,34 +2273,34 @@
       <c r="H2" s="2"/>
     </row>
     <row r="3" spans="1:12">
-      <c r="A3" s="164" t="s">
+      <c r="A3" s="148" t="s">
         <v>104</v>
       </c>
-      <c r="B3" s="164"/>
-      <c r="C3" s="164"/>
-      <c r="D3" s="164"/>
-      <c r="E3" s="164"/>
-      <c r="F3" s="164"/>
-      <c r="G3" s="164"/>
-      <c r="H3" s="164"/>
-      <c r="I3" s="164"/>
-      <c r="J3" s="164"/>
-      <c r="K3" s="164"/>
-      <c r="L3" s="164"/>
+      <c r="B3" s="148"/>
+      <c r="C3" s="148"/>
+      <c r="D3" s="148"/>
+      <c r="E3" s="148"/>
+      <c r="F3" s="148"/>
+      <c r="G3" s="148"/>
+      <c r="H3" s="148"/>
+      <c r="I3" s="148"/>
+      <c r="J3" s="148"/>
+      <c r="K3" s="148"/>
+      <c r="L3" s="148"/>
     </row>
     <row r="4" spans="1:12" ht="38.25" customHeight="1">
-      <c r="A4" s="164"/>
-      <c r="B4" s="164"/>
-      <c r="C4" s="164"/>
-      <c r="D4" s="164"/>
-      <c r="E4" s="164"/>
-      <c r="F4" s="164"/>
-      <c r="G4" s="164"/>
-      <c r="H4" s="164"/>
-      <c r="I4" s="164"/>
-      <c r="J4" s="164"/>
-      <c r="K4" s="164"/>
-      <c r="L4" s="164"/>
+      <c r="A4" s="148"/>
+      <c r="B4" s="148"/>
+      <c r="C4" s="148"/>
+      <c r="D4" s="148"/>
+      <c r="E4" s="148"/>
+      <c r="F4" s="148"/>
+      <c r="G4" s="148"/>
+      <c r="H4" s="148"/>
+      <c r="I4" s="148"/>
+      <c r="J4" s="148"/>
+      <c r="K4" s="148"/>
+      <c r="L4" s="148"/>
     </row>
     <row r="6" spans="1:12" ht="57" customHeight="1" thickBot="1">
       <c r="A6" s="4"/>
@@ -2765,9 +2761,9 @@
       <c r="L19" s="19"/>
     </row>
     <row r="20" spans="1:12" ht="57.75" customHeight="1" thickBot="1">
-      <c r="A20" s="165"/>
-      <c r="B20" s="165"/>
-      <c r="C20" s="165"/>
+      <c r="A20" s="149"/>
+      <c r="B20" s="149"/>
+      <c r="C20" s="149"/>
       <c r="D20" s="5" t="s">
         <v>0</v>
       </c>
@@ -2797,11 +2793,11 @@
       </c>
     </row>
     <row r="21" spans="1:12">
-      <c r="A21" s="151" t="s">
+      <c r="A21" s="150" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="151"/>
-      <c r="C21" s="151"/>
+      <c r="B21" s="150"/>
+      <c r="C21" s="150"/>
       <c r="D21" s="21"/>
       <c r="E21" s="21"/>
       <c r="F21" s="21"/>
@@ -3309,16 +3305,16 @@
       <c r="L37" s="40"/>
     </row>
     <row r="38" spans="1:12">
-      <c r="A38" s="154" t="s">
+      <c r="A38" s="151" t="s">
         <v>35</v>
       </c>
-      <c r="B38" s="154"/>
-      <c r="C38" s="154"/>
-      <c r="D38" s="154"/>
-      <c r="E38" s="154"/>
-      <c r="F38" s="154"/>
-      <c r="G38" s="154"/>
-      <c r="H38" s="154"/>
+      <c r="B38" s="151"/>
+      <c r="C38" s="151"/>
+      <c r="D38" s="151"/>
+      <c r="E38" s="151"/>
+      <c r="F38" s="151"/>
+      <c r="G38" s="151"/>
+      <c r="H38" s="151"/>
       <c r="I38" s="41"/>
       <c r="J38" s="42"/>
       <c r="K38" s="42"/>
@@ -3558,7 +3554,7 @@
         <v>-28.318584070796462</v>
       </c>
     </row>
-    <row r="46" spans="1:12" ht="24">
+    <row r="46" spans="1:12" ht="22">
       <c r="A46" s="45"/>
       <c r="B46" s="46" t="s">
         <v>39</v>
@@ -3594,7 +3590,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="47" spans="1:12" ht="24">
+    <row r="47" spans="1:12" ht="22">
       <c r="A47" s="45"/>
       <c r="B47" s="46" t="s">
         <v>40</v>
@@ -3645,12 +3641,12 @@
       <c r="L48" s="52"/>
     </row>
     <row r="49" spans="1:12">
-      <c r="A49" s="154" t="s">
+      <c r="A49" s="151" t="s">
         <v>41</v>
       </c>
-      <c r="B49" s="154"/>
-      <c r="C49" s="154"/>
-      <c r="D49" s="154"/>
+      <c r="B49" s="151"/>
+      <c r="C49" s="151"/>
+      <c r="D49" s="151"/>
       <c r="E49" s="53"/>
       <c r="F49" s="53"/>
       <c r="G49" s="49"/>
@@ -3749,12 +3745,12 @@
       <c r="L52" s="33"/>
     </row>
     <row r="53" spans="1:12">
-      <c r="A53" s="160" t="s">
+      <c r="A53" s="152" t="s">
         <v>44</v>
       </c>
-      <c r="B53" s="160"/>
-      <c r="C53" s="160"/>
-      <c r="D53" s="160"/>
+      <c r="B53" s="152"/>
+      <c r="C53" s="152"/>
+      <c r="D53" s="152"/>
       <c r="E53" s="53"/>
       <c r="F53" s="53"/>
       <c r="G53" s="49"/>
@@ -3972,7 +3968,7 @@
       <c r="K60" s="19"/>
       <c r="L60" s="19"/>
     </row>
-    <row r="61" spans="1:12" ht="48.6" thickBot="1">
+    <row r="61" spans="1:12" ht="43.5" thickBot="1">
       <c r="A61" s="4"/>
       <c r="B61" s="5"/>
       <c r="C61" s="5"/>
@@ -4323,12 +4319,12 @@
       <c r="L71" s="30"/>
     </row>
     <row r="72" spans="1:12">
-      <c r="A72" s="161" t="s">
+      <c r="A72" s="153" t="s">
         <v>49</v>
       </c>
-      <c r="B72" s="162"/>
-      <c r="C72" s="162"/>
-      <c r="D72" s="162"/>
+      <c r="B72" s="154"/>
+      <c r="C72" s="154"/>
+      <c r="D72" s="154"/>
       <c r="E72" s="53"/>
       <c r="F72" s="53"/>
       <c r="G72" s="53"/>
@@ -4533,12 +4529,12 @@
       <c r="L78" s="48"/>
     </row>
     <row r="79" spans="1:12">
-      <c r="A79" s="154" t="s">
+      <c r="A79" s="151" t="s">
         <v>50</v>
       </c>
-      <c r="B79" s="154"/>
-      <c r="C79" s="154"/>
-      <c r="D79" s="154"/>
+      <c r="B79" s="151"/>
+      <c r="C79" s="151"/>
+      <c r="D79" s="151"/>
       <c r="E79" s="48"/>
       <c r="F79" s="48"/>
       <c r="G79" s="48"/>
@@ -4745,16 +4741,16 @@
       <c r="L85" s="26"/>
     </row>
     <row r="86" spans="1:12">
-      <c r="A86" s="163" t="s">
+      <c r="A86" s="155" t="s">
         <v>52</v>
       </c>
-      <c r="B86" s="163"/>
-      <c r="C86" s="163"/>
-      <c r="D86" s="163"/>
-      <c r="E86" s="163"/>
-      <c r="F86" s="163"/>
-      <c r="G86" s="163"/>
-      <c r="H86" s="163"/>
+      <c r="B86" s="155"/>
+      <c r="C86" s="155"/>
+      <c r="D86" s="155"/>
+      <c r="E86" s="155"/>
+      <c r="F86" s="155"/>
+      <c r="G86" s="155"/>
+      <c r="H86" s="155"/>
       <c r="I86" s="70"/>
       <c r="J86" s="26"/>
       <c r="K86" s="71"/>
@@ -5201,12 +5197,12 @@
       <c r="L100" s="50"/>
     </row>
     <row r="101" spans="1:12">
-      <c r="A101" s="154" t="s">
+      <c r="A101" s="151" t="s">
         <v>59</v>
       </c>
-      <c r="B101" s="154"/>
-      <c r="C101" s="154"/>
-      <c r="D101" s="154"/>
+      <c r="B101" s="151"/>
+      <c r="C101" s="151"/>
+      <c r="D101" s="151"/>
       <c r="E101" s="53"/>
       <c r="F101" s="53"/>
       <c r="G101" s="53"/>
@@ -5341,12 +5337,12 @@
       <c r="L105" s="26"/>
     </row>
     <row r="106" spans="1:12">
-      <c r="A106" s="154" t="s">
+      <c r="A106" s="151" t="s">
         <v>61</v>
       </c>
-      <c r="B106" s="154"/>
-      <c r="C106" s="154"/>
-      <c r="D106" s="154"/>
+      <c r="B106" s="151"/>
+      <c r="C106" s="151"/>
+      <c r="D106" s="151"/>
       <c r="E106" s="30"/>
       <c r="F106" s="30"/>
       <c r="G106" s="30"/>
@@ -5597,12 +5593,12 @@
       </c>
     </row>
     <row r="115" spans="1:12">
-      <c r="A115" s="151" t="s">
+      <c r="A115" s="150" t="s">
         <v>62</v>
       </c>
-      <c r="B115" s="151"/>
-      <c r="C115" s="151"/>
-      <c r="D115" s="151"/>
+      <c r="B115" s="150"/>
+      <c r="C115" s="150"/>
+      <c r="D115" s="150"/>
       <c r="E115" s="83"/>
       <c r="F115" s="83"/>
       <c r="G115" s="83"/>
@@ -5989,16 +5985,16 @@
       <c r="L126" s="86"/>
     </row>
     <row r="127" spans="1:12">
-      <c r="A127" s="155" t="s">
+      <c r="A127" s="157" t="s">
         <v>70</v>
       </c>
-      <c r="B127" s="156"/>
-      <c r="C127" s="156"/>
-      <c r="D127" s="156"/>
-      <c r="E127" s="156"/>
-      <c r="F127" s="156"/>
-      <c r="G127" s="156"/>
-      <c r="H127" s="156"/>
+      <c r="B127" s="158"/>
+      <c r="C127" s="158"/>
+      <c r="D127" s="158"/>
+      <c r="E127" s="158"/>
+      <c r="F127" s="158"/>
+      <c r="G127" s="158"/>
+      <c r="H127" s="158"/>
       <c r="I127" s="92"/>
       <c r="J127" s="94"/>
       <c r="K127" s="94"/>
@@ -6365,10 +6361,10 @@
       </c>
     </row>
     <row r="138" spans="1:12">
-      <c r="A138" s="157"/>
-      <c r="B138" s="157"/>
-      <c r="C138" s="157"/>
-      <c r="D138" s="157"/>
+      <c r="A138" s="159"/>
+      <c r="B138" s="159"/>
+      <c r="C138" s="159"/>
+      <c r="D138" s="159"/>
       <c r="E138" s="104"/>
       <c r="F138" s="104"/>
       <c r="G138" s="104"/>
@@ -6379,12 +6375,12 @@
       <c r="L138" s="104"/>
     </row>
     <row r="139" spans="1:12">
-      <c r="A139" s="152" t="s">
+      <c r="A139" s="156" t="s">
         <v>71</v>
       </c>
-      <c r="B139" s="152"/>
-      <c r="C139" s="152"/>
-      <c r="D139" s="152"/>
+      <c r="B139" s="156"/>
+      <c r="C139" s="156"/>
+      <c r="D139" s="156"/>
       <c r="E139" s="104"/>
       <c r="F139" s="104"/>
       <c r="G139" s="104"/>
@@ -6481,12 +6477,12 @@
       <c r="L142" s="86"/>
     </row>
     <row r="143" spans="1:12">
-      <c r="A143" s="158" t="s">
+      <c r="A143" s="160" t="s">
         <v>74</v>
       </c>
-      <c r="B143" s="159"/>
-      <c r="C143" s="159"/>
-      <c r="D143" s="159"/>
+      <c r="B143" s="161"/>
+      <c r="C143" s="161"/>
+      <c r="D143" s="161"/>
       <c r="E143" s="86"/>
       <c r="F143" s="86"/>
       <c r="G143" s="86"/>
@@ -6635,12 +6631,12 @@
       <c r="L148" s="89"/>
     </row>
     <row r="149" spans="1:12">
-      <c r="A149" s="152" t="s">
+      <c r="A149" s="156" t="s">
         <v>77</v>
       </c>
-      <c r="B149" s="152"/>
-      <c r="C149" s="152"/>
-      <c r="D149" s="152"/>
+      <c r="B149" s="156"/>
+      <c r="C149" s="156"/>
+      <c r="D149" s="156"/>
       <c r="E149" s="86"/>
       <c r="F149" s="86"/>
       <c r="G149" s="86"/>
@@ -7098,7 +7094,7 @@
       <c r="K164" s="19"/>
       <c r="L164" s="19"/>
     </row>
-    <row r="165" spans="1:12" ht="48.6" thickBot="1">
+    <row r="165" spans="1:12" ht="43.5" thickBot="1">
       <c r="A165" s="4"/>
       <c r="B165" s="5"/>
       <c r="C165" s="5"/>
@@ -7131,16 +7127,16 @@
       </c>
     </row>
     <row r="166" spans="1:12">
-      <c r="A166" s="151" t="s">
+      <c r="A166" s="150" t="s">
         <v>80</v>
       </c>
-      <c r="B166" s="151"/>
-      <c r="C166" s="151"/>
-      <c r="D166" s="151"/>
-      <c r="E166" s="151"/>
-      <c r="F166" s="151"/>
-      <c r="G166" s="151"/>
-      <c r="H166" s="151"/>
+      <c r="B166" s="150"/>
+      <c r="C166" s="150"/>
+      <c r="D166" s="150"/>
+      <c r="E166" s="150"/>
+      <c r="F166" s="150"/>
+      <c r="G166" s="150"/>
+      <c r="H166" s="150"/>
       <c r="I166" s="124"/>
       <c r="J166" s="21"/>
       <c r="K166" s="21"/>
@@ -7233,16 +7229,16 @@
       <c r="L169" s="129"/>
     </row>
     <row r="170" spans="1:12">
-      <c r="A170" s="152" t="s">
+      <c r="A170" s="156" t="s">
         <v>82</v>
       </c>
-      <c r="B170" s="152"/>
-      <c r="C170" s="152"/>
-      <c r="D170" s="152"/>
-      <c r="E170" s="152"/>
-      <c r="F170" s="152"/>
-      <c r="G170" s="152"/>
-      <c r="H170" s="152"/>
+      <c r="B170" s="156"/>
+      <c r="C170" s="156"/>
+      <c r="D170" s="156"/>
+      <c r="E170" s="156"/>
+      <c r="F170" s="156"/>
+      <c r="G170" s="156"/>
+      <c r="H170" s="156"/>
       <c r="I170" s="131"/>
       <c r="J170" s="126"/>
       <c r="K170" s="129"/>
@@ -7348,7 +7344,7 @@
       <c r="K174" s="19"/>
       <c r="L174" s="19"/>
     </row>
-    <row r="175" spans="1:12" ht="48.6" thickBot="1">
+    <row r="175" spans="1:12" ht="43.5" thickBot="1">
       <c r="A175" s="4"/>
       <c r="B175" s="5"/>
       <c r="C175" s="5"/>
@@ -7381,10 +7377,10 @@
       </c>
     </row>
     <row r="176" spans="1:12">
-      <c r="A176" s="153" t="s">
+      <c r="A176" s="165" t="s">
         <v>83</v>
       </c>
-      <c r="B176" s="153"/>
+      <c r="B176" s="165"/>
       <c r="C176" s="9" t="s">
         <v>20</v>
       </c>
@@ -7417,10 +7413,10 @@
       </c>
     </row>
     <row r="177" spans="1:12">
-      <c r="A177" s="148" t="s">
+      <c r="A177" s="162" t="s">
         <v>84</v>
       </c>
-      <c r="B177" s="148"/>
+      <c r="B177" s="162"/>
       <c r="C177" s="135" t="s">
         <v>20</v>
       </c>
@@ -7453,10 +7449,10 @@
       </c>
     </row>
     <row r="178" spans="1:12">
-      <c r="A178" s="149" t="s">
+      <c r="A178" s="163" t="s">
         <v>19</v>
       </c>
-      <c r="B178" s="149"/>
+      <c r="B178" s="163"/>
       <c r="C178" s="140" t="s">
         <v>20</v>
       </c>
@@ -7503,10 +7499,10 @@
       <c r="L179" s="144"/>
     </row>
     <row r="180" spans="1:12">
-      <c r="A180" s="148" t="s">
+      <c r="A180" s="162" t="s">
         <v>85</v>
       </c>
-      <c r="B180" s="148"/>
+      <c r="B180" s="162"/>
       <c r="C180" s="135" t="s">
         <v>20</v>
       </c>
@@ -7539,10 +7535,10 @@
       </c>
     </row>
     <row r="181" spans="1:12">
-      <c r="A181" s="148" t="s">
+      <c r="A181" s="162" t="s">
         <v>86</v>
       </c>
-      <c r="B181" s="148"/>
+      <c r="B181" s="162"/>
       <c r="C181" s="135" t="s">
         <v>20</v>
       </c>
@@ -7575,10 +7571,10 @@
       </c>
     </row>
     <row r="182" spans="1:12">
-      <c r="A182" s="148" t="s">
+      <c r="A182" s="162" t="s">
         <v>87</v>
       </c>
-      <c r="B182" s="148"/>
+      <c r="B182" s="162"/>
       <c r="C182" s="135" t="s">
         <v>20</v>
       </c>
@@ -7611,10 +7607,10 @@
       </c>
     </row>
     <row r="183" spans="1:12">
-      <c r="A183" s="148" t="s">
+      <c r="A183" s="162" t="s">
         <v>88</v>
       </c>
-      <c r="B183" s="148"/>
+      <c r="B183" s="162"/>
       <c r="C183" s="135" t="s">
         <v>20</v>
       </c>
@@ -7647,10 +7643,10 @@
       </c>
     </row>
     <row r="184" spans="1:12">
-      <c r="A184" s="148" t="s">
+      <c r="A184" s="162" t="s">
         <v>89</v>
       </c>
-      <c r="B184" s="148"/>
+      <c r="B184" s="162"/>
       <c r="C184" s="135" t="s">
         <v>20</v>
       </c>
@@ -7683,10 +7679,10 @@
       </c>
     </row>
     <row r="185" spans="1:12">
-      <c r="A185" s="148" t="s">
+      <c r="A185" s="162" t="s">
         <v>90</v>
       </c>
-      <c r="B185" s="148"/>
+      <c r="B185" s="162"/>
       <c r="C185" s="135" t="s">
         <v>20</v>
       </c>
@@ -7719,10 +7715,10 @@
       </c>
     </row>
     <row r="186" spans="1:12">
-      <c r="A186" s="149" t="s">
+      <c r="A186" s="163" t="s">
         <v>21</v>
       </c>
-      <c r="B186" s="149"/>
+      <c r="B186" s="163"/>
       <c r="C186" s="140" t="s">
         <v>20</v>
       </c>
@@ -7755,10 +7751,10 @@
       </c>
     </row>
     <row r="187" spans="1:12">
-      <c r="A187" s="150" t="s">
+      <c r="A187" s="164" t="s">
         <v>91</v>
       </c>
-      <c r="B187" s="150"/>
+      <c r="B187" s="164"/>
       <c r="C187" s="86" t="s">
         <v>20</v>
       </c>
@@ -7818,7 +7814,7 @@
       <c r="K189" s="19"/>
       <c r="L189" s="19"/>
     </row>
-    <row r="190" spans="1:12" ht="48.6" thickBot="1">
+    <row r="190" spans="1:12" ht="43.5" thickBot="1">
       <c r="A190" s="4"/>
       <c r="B190" s="5"/>
       <c r="C190" s="5"/>
@@ -7851,10 +7847,10 @@
       </c>
     </row>
     <row r="191" spans="1:12">
-      <c r="A191" s="151" t="s">
+      <c r="A191" s="150" t="s">
         <v>92</v>
       </c>
-      <c r="B191" s="151"/>
+      <c r="B191" s="150"/>
       <c r="C191" s="19"/>
       <c r="D191" s="9"/>
       <c r="E191" s="9"/>
@@ -8562,23 +8558,6 @@
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="A3:L4"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="A38:H38"/>
-    <mergeCell ref="A49:D49"/>
-    <mergeCell ref="A53:D53"/>
-    <mergeCell ref="A72:D72"/>
-    <mergeCell ref="A79:D79"/>
-    <mergeCell ref="A86:H86"/>
-    <mergeCell ref="A101:D101"/>
-    <mergeCell ref="A106:D106"/>
-    <mergeCell ref="A149:D149"/>
-    <mergeCell ref="A115:D115"/>
-    <mergeCell ref="A127:H127"/>
-    <mergeCell ref="A138:D138"/>
-    <mergeCell ref="A139:D139"/>
-    <mergeCell ref="A143:D143"/>
     <mergeCell ref="A185:B185"/>
     <mergeCell ref="A186:B186"/>
     <mergeCell ref="A187:B187"/>
@@ -8593,6 +8572,23 @@
     <mergeCell ref="A181:B181"/>
     <mergeCell ref="A182:B182"/>
     <mergeCell ref="A183:B183"/>
+    <mergeCell ref="A106:D106"/>
+    <mergeCell ref="A149:D149"/>
+    <mergeCell ref="A115:D115"/>
+    <mergeCell ref="A127:H127"/>
+    <mergeCell ref="A138:D138"/>
+    <mergeCell ref="A139:D139"/>
+    <mergeCell ref="A143:D143"/>
+    <mergeCell ref="A53:D53"/>
+    <mergeCell ref="A72:D72"/>
+    <mergeCell ref="A79:D79"/>
+    <mergeCell ref="A86:H86"/>
+    <mergeCell ref="A101:D101"/>
+    <mergeCell ref="A3:L4"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A38:H38"/>
+    <mergeCell ref="A49:D49"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="56" fitToHeight="0" orientation="portrait" r:id="rId1"/>

</xml_diff>